<commit_message>
Changed two files: - `testing/moderation_goldens_v1/testcases_reviewed_v3.xlsx` - `testing/moderation_goldens_v1/testcases_reviewed_v3_semicolon.csv
</commit_message>
<xml_diff>
--- a/testing/moderation_goldens_v1/testcases_reviewed_v3.xlsx
+++ b/testing/moderation_goldens_v1/testcases_reviewed_v3.xlsx
@@ -548,14 +548,14 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Portrait</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>safe image</t>
@@ -583,7 +583,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Volgens Artes-productgrenzen: volledig gecoverd, safety = safe, geen sensitive overlay. Thema kan eventueel los als boudoir-discussie spelen, maar safety-uitkomst blijft safe.</t>
+          <t>Volgens Artes-productgrenzen: volledig gecoverd, safety = safe, geen sensitive overlay. Thema voor deze moderatiecase bewust gezet op Portrait zodat de publishflow de AI-call bereikt zonder boudoir-label.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harden Gemini adult boundaries and goldens
</commit_message>
<xml_diff>
--- a/testing/moderation_goldens_v1/testcases_reviewed_v3.xlsx
+++ b/testing/moderation_goldens_v1/testcases_reviewed_v3.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testcases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Testcases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Testcases'!$A$1:$M$5</definedName>
@@ -523,17 +523,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SAFE_01</t>
+          <t>ADULT_BDSM_01</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>images/safe/SAFE_01.jpg</t>
+          <t>images/adult/ADULT_BDSM_01.jpg</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -553,37 +553,37 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>18+ BDSM / kink</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>safe image</t>
+          <t>covered BDSM/kink without nudity or explicit sexual act</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>allowed</t>
+          <t>adult_context</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>allowed</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>allowed</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>visible without block</t>
+          <t>visible only with active 18+ entitlement</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Volgens Artes-productgrenzen: volledig gecoverd, safety = safe, geen sensitive overlay. Thema voor deze moderatiecase bewust gezet op Portrait zodat de publishflow de AI-call bereikt zonder boudoir-label.</t>
+          <t>Policy v2 correction after non-production live classifier inspection: this legacy SAFE_01 image contains covered BDSM/kink context. It is adult via erotic/kink triggers, but adultDecision must remain none because no nudity or explicit sexual act is visible.</t>
         </is>
       </c>
     </row>
@@ -697,27 +697,27 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>adult_nudity</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>review_required</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>visible as review or held state</t>
+          <t>visible only with active 18+ entitlement</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Volgens Artes-productgrenzen: geen boudoir, wel art nude. Zichtbare genitalien zonder duidelijke seksuele handeling. Dit type case hoort naar review om de grens binnen art nude te testen.</t>
+          <t>Policy v2 correction: visible genitalia without a visible sexual act is adult nudity, not explicit sexual content and not automatically review. Human review is reserved for genuine safety or explicit-act uncertainty.</t>
         </is>
       </c>
     </row>

</xml_diff>